<commit_message>
Fix Expected Result for CALL/SMS/USSD to be blank in template
ADB only confirms the intent was launched ("Starting: Intent {...}"),
not that the call connected. Blank Expected Result means any successful
launch is treated as PASS. GET_CONFIG still supports value matching.

https://claude.ai/code/session_01NVqk8RLBqGhSAEfLDYvE8o
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +40,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,15 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -437,7 +429,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -525,31 +517,11 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Call connects</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>(dry-run)</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Dry-run mode</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04 03:21:27</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -564,7 +536,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Phone2</t>
+          <t>Phone1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -577,31 +549,11 @@
           <t>Hello world</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>SMS composer opens</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>(dry-run)</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Dry-run mode</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04 03:21:27</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -625,31 +577,11 @@
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>USSD dialog appears</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>(dry-run)</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Dry-run mode</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04 03:21:27</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -677,31 +609,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Setting changed</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>(dry-run)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Dry-run mode</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04 03:21:27</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -727,29 +639,13 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Returns '1'</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>(dry-run)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>SKIP</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Dry-run mode</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-04 03:21:27</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>